<commit_message>
Cập nhật file excel từ bản đồ
</commit_message>
<xml_diff>
--- a/data/khaosat.xlsx
+++ b/data/khaosat.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O39"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2168,10 +2168,57 @@
       <c r="L38" t="str">
         <v/>
       </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
+        <v/>
+      </c>
+      <c r="O38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v/>
+      </c>
+      <c r="B39" t="str">
+        <v>home</v>
+      </c>
+      <c r="C39">
+        <v>10.760240950799044</v>
+      </c>
+      <c r="D39">
+        <v>106.61353282563975</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39">
+        <v>7</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
+      <c r="L39" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>